<commit_message>
Fix reserved metadata name in audit XLSForm
</commit_message>
<xml_diff>
--- a/docs/sentinel_project_audit_v2.xlsx
+++ b/docs/sentinel_project_audit_v2.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="survey" sheetId="1" r:id="R7bae12f7ab7c4d22"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="settings" sheetId="2" r:id="R859ccaca2afd422c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="survey" sheetId="1" r:id="R6e3ee384f5b643fe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="settings" sheetId="2" r:id="Re312f3955b094e34"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -256,12 +256,12 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="8.329999923706055" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="3.3299999237060547" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="17.440000534057617" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="22.670000076293945" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="5.889999866485596" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="6.21999979019165" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="14.220000267028809" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="7.440000057220459" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -553,50 +553,6 @@
       <x:c r="D20" s="1" t="str"/>
       <x:c r="E20" s="1" t="str"/>
       <x:c r="F20" s="1" t="str"/>
-    </x:row>
-    <x:row r="21">
-      <x:c r="A21" s="1" t="str">
-        <x:v>begin group</x:v>
-      </x:c>
-      <x:c r="B21" s="1" t="str">
-        <x:v>meta</x:v>
-      </x:c>
-      <x:c r="C21" s="1" t="str">
-        <x:v>Metadata</x:v>
-      </x:c>
-      <x:c r="D21" s="1" t="str"/>
-      <x:c r="E21" s="1" t="str"/>
-      <x:c r="F21" s="1" t="str"/>
-    </x:row>
-    <x:row r="22">
-      <x:c r="A22" s="1" t="str">
-        <x:v>calculate</x:v>
-      </x:c>
-      <x:c r="B22" s="1" t="str">
-        <x:v>instanceID</x:v>
-      </x:c>
-      <x:c r="C22" s="1" t="str">
-        <x:v>Instance ID</x:v>
-      </x:c>
-      <x:c r="D22" s="1" t="str">
-        <x:v>yes</x:v>
-      </x:c>
-      <x:c r="E22" s="1" t="str">
-        <x:v>yes</x:v>
-      </x:c>
-      <x:c r="F22" s="1" t="str">
-        <x:v>concat('uuid:', uuid())</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="23">
-      <x:c r="A23" s="1" t="str">
-        <x:v>end group</x:v>
-      </x:c>
-      <x:c r="B23" s="1" t="str"/>
-      <x:c r="C23" s="1" t="str"/>
-      <x:c r="D23" s="1" t="str"/>
-      <x:c r="E23" s="1" t="str"/>
-      <x:c r="F23" s="1" t="str"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Fix XLSForm settings layout
</commit_message>
<xml_diff>
--- a/docs/sentinel_project_audit_v2.xlsx
+++ b/docs/sentinel_project_audit_v2.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="survey" sheetId="1" r:id="R6e3ee384f5b643fe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="settings" sheetId="2" r:id="Re312f3955b094e34"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="survey" sheetId="1" r:id="Redd5b47441d24550"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="settings" sheetId="2" r:id="R8e28cf10ac034463"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -563,8 +563,10 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="10.5600004196167" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="32.66999816894531" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="14.670000076293945" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="14.890000343322754" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="5.21999979019165" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="32.66999816894531" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -572,30 +574,26 @@
         <x:v>form_title</x:v>
       </x:c>
       <x:c r="B1" s="3" t="str">
-        <x:v>Sentinel Project Audit</x:v>
+        <x:v>form_id</x:v>
+      </x:c>
+      <x:c r="C1" s="3" t="str">
+        <x:v>version</x:v>
+      </x:c>
+      <x:c r="D1" s="3" t="str">
+        <x:v>instance_name</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="1" t="str">
-        <x:v>form_id</x:v>
+        <x:v>Sentinel Project Audit</x:v>
       </x:c>
       <x:c r="B2" s="1" t="str">
         <x:v>sentinel_project_audit</x:v>
       </x:c>
-    </x:row>
-    <x:row r="3">
-      <x:c r="A3" s="1" t="str">
-        <x:v>version</x:v>
-      </x:c>
-      <x:c r="B3" s="1" t="str">
+      <x:c r="C2" s="1" t="str">
         <x:v>2</x:v>
       </x:c>
-    </x:row>
-    <x:row r="4">
-      <x:c r="A4" s="1" t="str">
-        <x:v>instance_name</x:v>
-      </x:c>
-      <x:c r="B4" s="1" t="str">
+      <x:c r="D2" s="1" t="str">
         <x:v>concat(${record_type}, ' ', ${source_instance_id})</x:v>
       </x:c>
     </x:row>

</xml_diff>